<commit_message>
Update 34Cl ENS flags and spreadsheet
Adjusts adopted-level annotations and DP status flags in A34/Cl34/new/Cl34_35k_ecp_decay_178_ms.ens: change DPE tag from R to C in header, allow E(p) from either 1980Ew02 or 2019ChZU, update several DP entries' status codes (R -> C or A ?), and add DPFLAG=A. Also updates the binary spreadsheet A35/K35/raw/35K EC, 36Ca ECP.xlsx (content changed).
</commit_message>
<xml_diff>
--- a/A35/K35/raw/35K EC, 36Ca ECP.xlsx
+++ b/A35/K35/raw/35K EC, 36Ca ECP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\A35\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\A35\K35\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE7BA670-BC27-4284-A058-9795CA2CB80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9206BD96-B68C-43B5-A978-42A93F598BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="2" xr2:uid="{80E8E01B-A04B-4992-8B74-8F4DE158A446}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{80E8E01B-A04B-4992-8B74-8F4DE158A446}"/>
   </bookViews>
   <sheets>
     <sheet name="36Ca" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="124">
   <si>
     <t>Ip</t>
   </si>
@@ -402,15 +405,23 @@
   </si>
   <si>
     <t>Table 3</t>
+  </si>
+  <si>
+    <t>ΣIp(rel)</t>
+  </si>
+  <si>
+    <t>DIp(abs)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
+    <numFmt numFmtId="178" formatCode="0.0%"/>
+    <numFmt numFmtId="181" formatCode="0.0000"/>
   </numFmts>
   <fonts count="24" x14ac:knownFonts="1">
     <font>
@@ -574,11 +585,20 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -587,7 +607,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -661,9 +681,6 @@
     <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -718,19 +735,46 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2549,503 +2593,712 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82375D98-27FE-4F56-B80A-6CBF87E329ED}">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="3" width="8.88671875" style="16"/>
-    <col min="4" max="4" width="10.44140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="9" width="8.88671875" style="16"/>
-    <col min="10" max="10" width="6.5546875" style="16" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="16"/>
+    <col min="1" max="4" width="8.88671875" style="16"/>
+    <col min="5" max="5" width="10.44140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="13" width="8.88671875" style="16"/>
+    <col min="14" max="14" width="6.5546875" style="16" customWidth="1"/>
+    <col min="15" max="16" width="8.88671875" style="16"/>
+    <col min="17" max="18" width="5.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.88671875" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="F1" s="16" t="s">
         <v>15</v>
       </c>
       <c r="G1" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="H1" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="I1" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="H1" s="16" t="s">
-        <v>119</v>
-      </c>
-      <c r="I1" s="16" t="s">
+      <c r="L1" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="M1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="O1" s="16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="20">
         <v>665.56</v>
       </c>
-      <c r="B2" s="21">
-        <f>I2-A16-A2</f>
+      <c r="B2" s="20"/>
+      <c r="C2" s="21">
+        <f>M2-A16-A2</f>
         <v>965.24000000000024</v>
       </c>
-      <c r="C2" s="20">
+      <c r="D2" s="20">
         <v>11</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="E2" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="I2" s="20">
+      <c r="M2" s="20">
         <v>7527</v>
       </c>
-      <c r="J2" s="20">
+      <c r="N2" s="20">
         <v>11</v>
       </c>
-      <c r="K2" s="20" t="s">
+      <c r="O2" s="20" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B3" s="16">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="B3" s="19">
+        <f>C3/35*34</f>
+        <v>1282.2857142857142</v>
+      </c>
+      <c r="C3" s="16">
         <v>1320</v>
       </c>
-      <c r="C3" s="16">
+      <c r="D3" s="16">
         <v>20</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="E3" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="16">
+      <c r="F3" s="16">
         <v>16</v>
       </c>
-      <c r="F3" s="16">
+      <c r="G3" s="16">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J3" s="19">
+        <v>1282.2857142857142</v>
+      </c>
+      <c r="K3" s="46">
+        <f>F3*O$16</f>
+        <v>1.6959999999999999E-2</v>
+      </c>
+      <c r="L3" s="46">
+        <f>K3*0.4</f>
+        <v>6.7840000000000001E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="20">
         <v>146.36000000000001</v>
       </c>
-      <c r="B4" s="20">
+      <c r="B4" s="19">
+        <f t="shared" ref="B4:B12" si="0">C4/35*34</f>
+        <v>1425.0857142857142</v>
+      </c>
+      <c r="C4" s="20">
         <v>1467</v>
       </c>
-      <c r="C4" s="20">
+      <c r="D4" s="20">
         <v>20</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="E4" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="20">
+      <c r="F4" s="20">
         <v>100</v>
       </c>
-      <c r="F4" s="20">
+      <c r="G4" s="20">
         <v>8</v>
       </c>
-      <c r="G4" s="20">
-        <f>E4+E5</f>
+      <c r="H4" s="20">
+        <f>F4+F5</f>
         <v>141</v>
       </c>
-      <c r="H4" s="20">
-        <f>SQRT(SUMSQ(F4+F5+F6))</f>
+      <c r="I4" s="20">
+        <f>SQRT(SUMSQ(G4+G5+G6))</f>
         <v>19</v>
       </c>
-      <c r="I4" s="21">
-        <f>B4+A4+$A$16</f>
+      <c r="J4" s="21">
+        <v>1425.0857142857142</v>
+      </c>
+      <c r="K4" s="46">
+        <f>F4*O$16</f>
+        <v>0.106</v>
+      </c>
+      <c r="L4" s="46">
+        <f t="shared" ref="L4:L13" si="1">K4*0.4</f>
+        <v>4.24E-2</v>
+      </c>
+      <c r="M4" s="21">
+        <f>C4+A4+$A$16</f>
         <v>7509.5599999999995</v>
       </c>
-      <c r="J4" s="21">
-        <f>C4</f>
+      <c r="N4" s="21">
+        <f>D4</f>
         <v>20</v>
       </c>
-      <c r="K4" s="20">
+      <c r="O4" s="20">
         <v>7504</v>
       </c>
-      <c r="L4" s="20">
+      <c r="P4" s="20">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="20">
         <v>0</v>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="19">
+        <f t="shared" si="0"/>
+        <v>1555.2571428571428</v>
+      </c>
+      <c r="C5" s="20">
         <v>1601</v>
       </c>
-      <c r="C5" s="20">
+      <c r="D5" s="20">
         <v>20</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="E5" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="20">
+      <c r="F5" s="20">
         <v>41</v>
       </c>
-      <c r="F5" s="20">
+      <c r="G5" s="20">
         <v>5</v>
       </c>
-      <c r="G5" s="20"/>
       <c r="H5" s="20"/>
-      <c r="I5" s="21">
-        <f>B5+A5+$A$16</f>
+      <c r="I5" s="20"/>
+      <c r="J5" s="21">
+        <v>1555.2571428571428</v>
+      </c>
+      <c r="K5" s="46">
+        <f>F5*O$16</f>
+        <v>4.3459999999999999E-2</v>
+      </c>
+      <c r="L5" s="46">
+        <f t="shared" si="1"/>
+        <v>1.7384E-2</v>
+      </c>
+      <c r="M5" s="21">
+        <f>C5+A5+$A$16</f>
         <v>7497.2</v>
       </c>
-      <c r="J5" s="21">
-        <f t="shared" ref="J5" si="0">C5</f>
+      <c r="N5" s="21">
+        <f t="shared" ref="N5" si="2">D5</f>
         <v>20</v>
       </c>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B6" s="16">
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="B6" s="19">
+        <f t="shared" si="0"/>
+        <v>1704.8571428571429</v>
+      </c>
+      <c r="C6" s="16">
         <v>1755</v>
       </c>
-      <c r="C6" s="16">
+      <c r="D6" s="16">
         <v>20</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="E6" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="16">
+      <c r="F6" s="16">
         <v>42</v>
       </c>
-      <c r="F6" s="16">
+      <c r="G6" s="16">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B7" s="16">
+      <c r="J6" s="19">
+        <v>1704.8571428571429</v>
+      </c>
+      <c r="K6" s="46">
+        <f>F6*O$16</f>
+        <v>4.4519999999999997E-2</v>
+      </c>
+      <c r="L6" s="46">
+        <f t="shared" si="1"/>
+        <v>1.7808000000000001E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="B7" s="19">
+        <f t="shared" si="0"/>
+        <v>1874.8571428571429</v>
+      </c>
+      <c r="C7" s="16">
         <v>1930</v>
       </c>
-      <c r="C7" s="16">
+      <c r="D7" s="16">
         <v>20</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="E7" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="16">
+      <c r="F7" s="16">
         <v>24</v>
       </c>
-      <c r="F7" s="16">
+      <c r="G7" s="16">
         <v>4</v>
       </c>
-      <c r="K7" s="16" t="s">
+      <c r="J7" s="19">
+        <v>1874.8571428571429</v>
+      </c>
+      <c r="K7" s="46">
+        <f>F7*O$16</f>
+        <v>2.5439999999999997E-2</v>
+      </c>
+      <c r="L7" s="46">
+        <f t="shared" si="1"/>
+        <v>1.0175999999999999E-2</v>
+      </c>
+      <c r="O7" s="16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="22">
         <v>461</v>
       </c>
-      <c r="B8" s="23">
+      <c r="B8" s="19">
+        <f t="shared" si="0"/>
+        <v>1979.7714285714285</v>
+      </c>
+      <c r="C8" s="23">
         <v>2038</v>
       </c>
-      <c r="C8" s="23">
+      <c r="D8" s="23">
         <v>20</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="E8" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="23">
+      <c r="F8" s="23">
         <v>17</v>
       </c>
-      <c r="F8" s="23">
+      <c r="G8" s="23">
         <v>3</v>
       </c>
-      <c r="G8" s="23">
-        <f>E8+E9+E10</f>
+      <c r="H8" s="23">
+        <f>F8+F9+F10</f>
         <v>59</v>
       </c>
-      <c r="H8" s="23">
-        <f>SQRT(SUMSQ(F8+F9+F10))</f>
+      <c r="I8" s="23">
+        <f>SQRT(SUMSQ(G8+G9+G10))</f>
         <v>11</v>
       </c>
-      <c r="I8" s="24">
-        <f>B8+A8+$A$16</f>
+      <c r="J8" s="24">
+        <v>1979.7714285714285</v>
+      </c>
+      <c r="K8" s="46">
+        <f>F8*O$16</f>
+        <v>1.8019999999999998E-2</v>
+      </c>
+      <c r="L8" s="46">
+        <f t="shared" si="1"/>
+        <v>7.2079999999999991E-3</v>
+      </c>
+      <c r="M8" s="24">
+        <f>C8+A8+$A$16</f>
         <v>8395.2000000000007</v>
       </c>
-      <c r="J8" s="24">
-        <f>C8</f>
+      <c r="N8" s="24">
+        <f>D8</f>
         <v>20</v>
       </c>
-      <c r="K8" s="23" t="s">
+      <c r="O8" s="23" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="23">
         <v>146.36000000000001</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="19">
+        <f t="shared" si="0"/>
+        <v>2281.8857142857141</v>
+      </c>
+      <c r="C9" s="23">
         <v>2349</v>
       </c>
-      <c r="C9" s="23">
+      <c r="D9" s="23">
         <v>20</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="E9" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="23">
+      <c r="F9" s="23">
         <v>23</v>
       </c>
-      <c r="F9" s="23">
+      <c r="G9" s="23">
         <v>4</v>
       </c>
-      <c r="G9" s="23"/>
       <c r="H9" s="23"/>
-      <c r="I9" s="24">
-        <f>B9+A9+$A$16</f>
+      <c r="I9" s="23"/>
+      <c r="J9" s="24">
+        <v>2281.8857142857141</v>
+      </c>
+      <c r="K9" s="46">
+        <f>F9*O$16</f>
+        <v>2.4379999999999999E-2</v>
+      </c>
+      <c r="L9" s="46">
+        <f t="shared" si="1"/>
+        <v>9.7520000000000003E-3</v>
+      </c>
+      <c r="M9" s="24">
+        <f>C9+A9+$A$16</f>
         <v>8391.56</v>
       </c>
-      <c r="J9" s="24">
-        <f t="shared" ref="J9:J10" si="1">C9</f>
+      <c r="N9" s="24">
+        <f t="shared" ref="N9:N10" si="3">D9</f>
         <v>20</v>
       </c>
-      <c r="K9" s="23"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O9" s="23"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="23">
         <v>0</v>
       </c>
-      <c r="B10" s="23">
+      <c r="B10" s="19">
+        <f t="shared" si="0"/>
+        <v>2424.6857142857143</v>
+      </c>
+      <c r="C10" s="23">
         <v>2496</v>
       </c>
-      <c r="C10" s="23">
+      <c r="D10" s="23">
         <v>20</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="E10" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="23">
+      <c r="F10" s="23">
         <v>19</v>
       </c>
-      <c r="F10" s="23">
+      <c r="G10" s="23">
         <v>4</v>
       </c>
-      <c r="G10" s="23"/>
       <c r="H10" s="23"/>
-      <c r="I10" s="24">
-        <f>B10+A10+$A$16</f>
+      <c r="I10" s="23"/>
+      <c r="J10" s="24">
+        <v>2424.6857142857143</v>
+      </c>
+      <c r="K10" s="46">
+        <f>F10*O$16</f>
+        <v>2.0139999999999998E-2</v>
+      </c>
+      <c r="L10" s="46">
+        <f t="shared" si="1"/>
+        <v>8.0559999999999989E-3</v>
+      </c>
+      <c r="M10" s="24">
+        <f>C10+A10+$A$16</f>
         <v>8392.2000000000007</v>
       </c>
-      <c r="J10" s="24">
+      <c r="N10" s="24">
+        <f t="shared" si="3"/>
+        <v>20</v>
+      </c>
+      <c r="O10" s="23"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="B11" s="19">
+        <f t="shared" si="0"/>
+        <v>2575.2571428571432</v>
+      </c>
+      <c r="C11" s="16">
+        <v>2651</v>
+      </c>
+      <c r="D11" s="16">
+        <v>20</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="16">
+        <v>10</v>
+      </c>
+      <c r="G11" s="16">
+        <v>3</v>
+      </c>
+      <c r="J11" s="19">
+        <v>2575.2571428571432</v>
+      </c>
+      <c r="K11" s="46">
+        <f>F11*O$16</f>
+        <v>1.06E-2</v>
+      </c>
+      <c r="L11" s="46">
         <f t="shared" si="1"/>
+        <v>4.2399999999999998E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="B12" s="19">
+        <f t="shared" si="0"/>
+        <v>2807.4285714285716</v>
+      </c>
+      <c r="C12" s="16">
+        <v>2890</v>
+      </c>
+      <c r="D12" s="16">
         <v>20</v>
       </c>
-      <c r="K10" s="23"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B11" s="16">
-        <v>2651</v>
-      </c>
-      <c r="C11" s="16">
-        <v>20</v>
-      </c>
-      <c r="D11" s="16" t="s">
+      <c r="E12" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="16">
-        <v>10</v>
-      </c>
-      <c r="F11" s="16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B12" s="16">
-        <v>2890</v>
-      </c>
-      <c r="C12" s="16">
-        <v>20</v>
-      </c>
-      <c r="D12" s="16" t="s">
+      <c r="F12" s="16">
+        <v>5.7</v>
+      </c>
+      <c r="G12" s="16">
+        <v>1.8</v>
+      </c>
+      <c r="J12" s="19">
+        <v>2807.4285714285716</v>
+      </c>
+      <c r="K12" s="46">
+        <f>F12*O$16</f>
+        <v>6.0419999999999996E-3</v>
+      </c>
+      <c r="L12" s="46">
+        <f t="shared" si="1"/>
+        <v>2.4168000000000002E-3</v>
+      </c>
+      <c r="M12" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="16">
-        <v>5.7</v>
-      </c>
-      <c r="F12" s="16">
-        <v>1.8</v>
-      </c>
-      <c r="I12" s="16" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="D13" s="16" t="s">
+    </row>
+    <row r="13" spans="1:18" s="53" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="E13" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="E13" s="43">
-        <f>SUM(E3:E12)</f>
+      <c r="F13" s="54">
+        <f>SUM(F3:F12)</f>
         <v>297.7</v>
       </c>
-      <c r="F13" s="17">
-        <f>SQRT(SUMSQ(F3:F12))</f>
+      <c r="G13" s="55">
+        <f>SQRT(SUMSQ(G3:G12))</f>
         <v>14.25622670975739</v>
       </c>
-      <c r="I13" s="16" t="s">
+      <c r="K13" s="56">
+        <f>F13*O$16</f>
+        <v>0.31556199999999995</v>
+      </c>
+      <c r="L13" s="56">
+        <f t="shared" si="1"/>
+        <v>0.1262248</v>
+      </c>
+      <c r="M13" s="53" t="s">
         <v>121</v>
       </c>
-      <c r="K13" s="16" t="s">
+      <c r="O13" s="53" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="D14" s="16" t="s">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="E14" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="25">
-        <v>3.7000000000000002E-3</v>
-      </c>
-      <c r="F14" s="25">
-        <v>1.5E-3</v>
-      </c>
-      <c r="G14" s="26">
-        <f>G8/$E$13*$E$14</f>
-        <v>7.3328854551561978E-4</v>
-      </c>
-      <c r="H14" s="26">
+      <c r="F14" s="49">
+        <v>0.37</v>
+      </c>
+      <c r="G14" s="49">
+        <v>0.15</v>
+      </c>
+      <c r="H14" s="47">
+        <f>H8/$F$13*$F$14</f>
+        <v>7.3328854551561976E-2</v>
+      </c>
+      <c r="I14" s="47">
         <v>3.1E-4</v>
       </c>
-      <c r="I14" s="45">
-        <f>0.062%</f>
-        <v>6.2E-4</v>
-      </c>
-      <c r="J14" s="44">
-        <v>2.5999999999999998E-4</v>
-      </c>
-      <c r="K14" s="46">
-        <f>I14/G14</f>
+      <c r="J14" s="47"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="25"/>
+      <c r="M14" s="50">
+        <v>6.2E-2</v>
+      </c>
+      <c r="N14" s="49">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="O14" s="43">
+        <f>M14/H14</f>
         <v>0.84550618415025192</v>
       </c>
-      <c r="L14" s="46">
-        <f>J14/H14</f>
-        <v>0.83870967741935476</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="P14" s="43">
+        <f>N14/I14</f>
+        <v>83.870967741935473</v>
+      </c>
+      <c r="Q14" s="45">
+        <f>N14/M14</f>
+        <v>0.41935483870967738</v>
+      </c>
+      <c r="R14" s="45">
+        <f>G14/F14</f>
+        <v>0.40540540540540537</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="27">
-        <f>(G4)/$E$13*$E$14</f>
-        <v>1.7524353375881761E-3</v>
-      </c>
-      <c r="H15" s="27">
+      <c r="H15" s="48">
+        <f>(H4)/$F$13*$F$14</f>
+        <v>0.1752435337588176</v>
+      </c>
+      <c r="I15" s="48">
         <v>6.9999999999999999E-4</v>
       </c>
-      <c r="I15" s="47">
-        <v>1.5E-3</v>
-      </c>
-      <c r="J15" s="25">
-        <v>5.9999999999999995E-4</v>
-      </c>
-      <c r="K15" s="48">
-        <f>I15/G15</f>
-        <v>0.85595169637722834</v>
-      </c>
-      <c r="L15" s="48">
-        <f>J15/H15</f>
-        <v>0.8571428571428571</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J15" s="48"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="26"/>
+      <c r="M15" s="51">
+        <v>0.15</v>
+      </c>
+      <c r="N15" s="49">
+        <v>0.06</v>
+      </c>
+      <c r="O15" s="44">
+        <f>M15/H15</f>
+        <v>0.85595169637722823</v>
+      </c>
+      <c r="P15" s="44">
+        <f>N15/I15</f>
+        <v>85.714285714285708</v>
+      </c>
+      <c r="Q15" s="45">
+        <f>N15/M15</f>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="12" x14ac:dyDescent="0.3">
       <c r="A16" s="16">
         <v>5896.2</v>
       </c>
-      <c r="B16" s="16">
+      <c r="C16" s="16">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H16" s="16">
+        <f>H4+H8</f>
+        <v>200</v>
+      </c>
+      <c r="M16" s="49">
+        <f>M14+M15</f>
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="N16" s="52">
+        <f>M16*0.4</f>
+        <v>8.48E-2</v>
+      </c>
+      <c r="O16" s="35">
+        <f>M16/H16</f>
+        <v>1.06E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E20" s="16">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F20" s="16">
         <v>5.4</v>
       </c>
-      <c r="F20" s="16">
+      <c r="G20" s="16">
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E21" s="16">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F21" s="16">
         <v>33.6</v>
       </c>
-      <c r="F21" s="16">
+      <c r="G21" s="16">
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E22" s="16">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F22" s="16">
         <v>13.8</v>
       </c>
-      <c r="F22" s="16">
+      <c r="G22" s="16">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E23" s="16">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F23" s="16">
         <v>14.1</v>
       </c>
-      <c r="F23" s="16">
+      <c r="G23" s="16">
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E24" s="16">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F24" s="16">
         <v>8.1</v>
       </c>
-      <c r="F24" s="16">
+      <c r="G24" s="16">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E25" s="16">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F25" s="16">
         <v>5.7</v>
       </c>
-      <c r="F25" s="16">
+      <c r="G25" s="16">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E26" s="16">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F26" s="16">
         <v>7.7</v>
       </c>
-      <c r="F26" s="16">
+      <c r="G26" s="16">
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E27" s="16">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F27" s="16">
         <v>6.4</v>
       </c>
-      <c r="F27" s="16">
+      <c r="G27" s="16">
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E28" s="16">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F28" s="16">
         <v>3.4</v>
       </c>
-      <c r="F28" s="16">
+      <c r="G28" s="16">
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E29" s="16">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F29" s="16">
         <v>1.9</v>
       </c>
-      <c r="F29" s="16">
+      <c r="G29" s="16">
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E30" s="16">
-        <f>SUM(E20:E29)</f>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F30" s="16">
+        <f>SUM(F20:F29)</f>
         <v>100.10000000000001</v>
       </c>
     </row>
@@ -3085,40 +3338,40 @@
       <c r="E1" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="F1" s="36">
+      <c r="F1" s="35">
         <f>F2</f>
         <v>83.6</v>
       </c>
-      <c r="G1" s="36">
+      <c r="G1" s="35">
         <f>G2</f>
         <v>0.5</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="D2" s="33" t="s">
+      <c r="D2" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="E2" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="F2" s="33">
+      <c r="F2" s="32">
         <v>83.6</v>
       </c>
-      <c r="G2" s="33">
+      <c r="G2" s="32">
         <v>0.5</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="D3" s="33" t="s">
+      <c r="D3" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="E3" s="33" t="s">
+      <c r="E3" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="F3" s="33">
+      <c r="F3" s="32">
         <v>78</v>
       </c>
-      <c r="G3" s="33">
+      <c r="G3" s="32">
         <v>20</v>
       </c>
       <c r="J3" s="16">
@@ -3280,15 +3533,15 @@
       </c>
       <c r="K7" s="19"/>
       <c r="L7" s="19"/>
-      <c r="M7" s="30">
-        <f t="shared" ref="M7:M19" si="3">MAX(I7:L7)</f>
+      <c r="M7" s="29">
+        <f t="shared" ref="M7:M17" si="3">MAX(I7:L7)</f>
         <v>4981.9058823529413</v>
       </c>
-      <c r="N7" s="30">
+      <c r="N7" s="29">
         <f t="shared" ref="N7:N19" si="4">SQRT($H7^2+G$1^2)</f>
         <v>13.39169034297816</v>
       </c>
-      <c r="O7" s="31" t="s">
+      <c r="O7" s="30" t="s">
         <v>89</v>
       </c>
       <c r="X7" s="17">
@@ -3570,15 +3823,15 @@
       <c r="J12" s="19"/>
       <c r="K12" s="19"/>
       <c r="L12" s="19"/>
-      <c r="M12" s="30">
+      <c r="M12" s="29">
         <f t="shared" si="3"/>
         <v>4977.4235294117643</v>
       </c>
-      <c r="N12" s="30">
+      <c r="N12" s="29">
         <f>SQRT($H12^2+G$1^2)</f>
         <v>39.120842417037558</v>
       </c>
-      <c r="O12" s="31" t="s">
+      <c r="O12" s="30" t="s">
         <v>89</v>
       </c>
       <c r="X12" s="17">
@@ -3697,13 +3950,13 @@
       <c r="O14" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="X14" s="43">
+      <c r="X14" s="42">
         <v>0.72</v>
       </c>
       <c r="Y14" s="16">
         <v>18</v>
       </c>
-      <c r="Z14" s="43">
+      <c r="Z14" s="42">
         <f t="shared" si="5"/>
         <v>0.71570576540755471</v>
       </c>
@@ -3755,13 +4008,13 @@
       <c r="O15" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="X15" s="43">
+      <c r="X15" s="42">
         <v>0.61</v>
       </c>
       <c r="Y15" s="16">
         <v>15</v>
       </c>
-      <c r="Z15" s="43">
+      <c r="Z15" s="42">
         <f t="shared" si="5"/>
         <v>0.60636182902584501</v>
       </c>
@@ -3813,13 +4066,13 @@
       <c r="O16" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="X16" s="43">
+      <c r="X16" s="42">
         <v>1.43</v>
       </c>
       <c r="Y16" s="16">
         <v>17</v>
       </c>
-      <c r="Z16" s="43">
+      <c r="Z16" s="42">
         <f t="shared" si="5"/>
         <v>1.4214711729622267</v>
       </c>
@@ -3871,13 +4124,13 @@
       <c r="O17" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="X17" s="43">
+      <c r="X17" s="42">
         <v>1.4</v>
       </c>
       <c r="Y17" s="16">
         <v>19</v>
       </c>
-      <c r="Z17" s="43">
+      <c r="Z17" s="42">
         <f t="shared" si="5"/>
         <v>1.3916500994035785</v>
       </c>
@@ -3916,18 +4169,18 @@
         <f>$F18+$F$1+J$5</f>
         <v>9157.2000000000007</v>
       </c>
-      <c r="M18" s="38">
+      <c r="M18" s="37">
         <f>MAX(I18:L18)</f>
         <v>9157.2000000000007</v>
       </c>
-      <c r="N18" s="38">
+      <c r="N18" s="37">
         <f t="shared" si="4"/>
         <v>22.652577631616261</v>
       </c>
-      <c r="O18" s="39" t="s">
+      <c r="O18" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="P18" s="39" t="s">
+      <c r="P18" s="38" t="s">
         <v>113</v>
       </c>
       <c r="X18" s="17">
@@ -3974,27 +4227,27 @@
         <f>$F19+$F$1</f>
         <v>9144.4823529411769</v>
       </c>
-      <c r="M19" s="38">
+      <c r="M19" s="37">
         <f>MAX(I19:L19)</f>
         <v>9144.4823529411769</v>
       </c>
-      <c r="N19" s="38">
+      <c r="N19" s="37">
         <f t="shared" si="4"/>
         <v>91.61901141463575</v>
       </c>
-      <c r="O19" s="39" t="s">
+      <c r="O19" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="P19" s="39" t="s">
+      <c r="P19" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="X19" s="43">
+      <c r="X19" s="42">
         <v>0.41</v>
       </c>
       <c r="Y19" s="16">
         <v>6</v>
       </c>
-      <c r="Z19" s="43">
+      <c r="Z19" s="42">
         <f t="shared" si="5"/>
         <v>0.4075546719681909</v>
       </c>
@@ -4006,7 +4259,7 @@
       <c r="I20" s="19"/>
       <c r="M20" s="19"/>
       <c r="N20" s="19"/>
-      <c r="X20" s="43"/>
+      <c r="X20" s="42"/>
       <c r="Z20" s="17"/>
     </row>
     <row r="21" spans="1:26" ht="13.2" x14ac:dyDescent="0.3">
@@ -4046,7 +4299,7 @@
       <c r="R21" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="X21" s="43">
+      <c r="X21" s="42">
         <v>2.2000000000000002</v>
       </c>
       <c r="Y21" s="16">
@@ -4094,13 +4347,13 @@
       <c r="R22" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="X22" s="43">
+      <c r="X22" s="42">
         <v>1.0900000000000001</v>
       </c>
       <c r="Y22" s="16">
         <v>17</v>
       </c>
-      <c r="Z22" s="43">
+      <c r="Z22" s="42">
         <f t="shared" ref="Z22:Z33" si="9">X22*100/100.6</f>
         <v>1.0834990059642149</v>
       </c>
@@ -4132,17 +4385,17 @@
         <v>7424.3352941176481</v>
       </c>
       <c r="J23" s="19"/>
-      <c r="P23" s="28">
+      <c r="P23" s="27">
         <f>MAX(I23:L23)</f>
         <v>7424.3352941176481</v>
       </c>
-      <c r="Q23" s="29" t="s">
+      <c r="Q23" s="28" t="s">
         <v>82</v>
       </c>
       <c r="R23" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="X23" s="43">
+      <c r="X23" s="42">
         <v>1.1000000000000001</v>
       </c>
       <c r="Y23" s="16">
@@ -4189,7 +4442,7 @@
         <f>R21</f>
         <v>L8</v>
       </c>
-      <c r="X24" s="43">
+      <c r="X24" s="42">
         <v>2.2000000000000002</v>
       </c>
       <c r="Y24" s="16">
@@ -4236,13 +4489,13 @@
         <f>R22</f>
         <v>L16</v>
       </c>
-      <c r="X25" s="43">
+      <c r="X25" s="42">
         <v>1.0900000000000001</v>
       </c>
       <c r="Y25" s="16">
         <v>17</v>
       </c>
-      <c r="Z25" s="43">
+      <c r="Z25" s="42">
         <f t="shared" si="9"/>
         <v>1.0834990059642149</v>
       </c>
@@ -4272,18 +4525,18 @@
         <f>$F26+$F$1</f>
         <v>8202.5705882352941</v>
       </c>
-      <c r="S26" s="28">
+      <c r="S26" s="27">
         <f>MAX(I26:L26)</f>
         <v>8202.5705882352941</v>
       </c>
-      <c r="T26" s="28" t="s">
+      <c r="T26" s="27" t="s">
         <v>83</v>
       </c>
       <c r="U26" s="16" t="str">
         <f>R23</f>
         <v>L17</v>
       </c>
-      <c r="X26" s="43">
+      <c r="X26" s="42">
         <v>1.1000000000000001</v>
       </c>
       <c r="Y26" s="16">
@@ -4307,7 +4560,7 @@
       <c r="D27" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="E27" s="42">
+      <c r="E27" s="41">
         <f>(LEFT(B21,4)+RIGHT(B21,4))/2</f>
         <v>3223.5</v>
       </c>
@@ -4321,18 +4574,18 @@
         <f>$F27+$F$1+J$5</f>
         <v>5493.0088235294115</v>
       </c>
-      <c r="M27" s="37">
+      <c r="M27" s="36">
         <f>MAX(I27:L27)</f>
         <v>5493.0088235294115</v>
       </c>
-      <c r="N27" s="37" t="s">
+      <c r="N27" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="O27" s="36" t="str">
+      <c r="O27" s="35" t="str">
         <f>R21</f>
         <v>L8</v>
       </c>
-      <c r="X27" s="43">
+      <c r="X27" s="42">
         <v>2.2000000000000002</v>
       </c>
       <c r="Y27" s="16">
@@ -4356,7 +4609,7 @@
       <c r="D28" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="E28" s="36">
+      <c r="E28" s="35">
         <f>(LEFT(B22,4)+RIGHT(B22,4))/2</f>
         <v>6316</v>
       </c>
@@ -4370,24 +4623,24 @@
         <v>6585.3647058823526</v>
       </c>
       <c r="J28" s="19"/>
-      <c r="M28" s="40">
+      <c r="M28" s="39">
         <f>MAX(I28:L28)</f>
         <v>6585.3647058823526</v>
       </c>
-      <c r="N28" s="40" t="s">
+      <c r="N28" s="39" t="s">
         <v>84</v>
       </c>
-      <c r="O28" s="36" t="str">
+      <c r="O28" s="35" t="str">
         <f>R22</f>
         <v>L16</v>
       </c>
-      <c r="X28" s="43">
+      <c r="X28" s="42">
         <v>1.0900000000000001</v>
       </c>
       <c r="Y28" s="16">
         <v>17</v>
       </c>
-      <c r="Z28" s="43">
+      <c r="Z28" s="42">
         <f t="shared" si="9"/>
         <v>1.0834990059642149</v>
       </c>
@@ -4405,7 +4658,7 @@
       <c r="D29" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="E29" s="36">
+      <c r="E29" s="35">
         <f>(LEFT(B23,4)+RIGHT(B23,4))/2</f>
         <v>7509</v>
       </c>
@@ -4419,18 +4672,18 @@
         <v>7813.4529411764706</v>
       </c>
       <c r="J29" s="19"/>
-      <c r="M29" s="41">
+      <c r="M29" s="40">
         <f>MAX(I29:L29)</f>
         <v>7813.4529411764706</v>
       </c>
-      <c r="N29" s="41" t="s">
+      <c r="N29" s="40" t="s">
         <v>84</v>
       </c>
-      <c r="O29" s="36" t="str">
+      <c r="O29" s="35" t="str">
         <f>R23</f>
         <v>L17</v>
       </c>
-      <c r="X29" s="43">
+      <c r="X29" s="42">
         <v>1.1000000000000001</v>
       </c>
       <c r="Y29" s="16">
@@ -4442,10 +4695,10 @@
       </c>
     </row>
     <row r="30" spans="1:26" ht="12" x14ac:dyDescent="0.3">
-      <c r="M30" s="36"/>
-      <c r="N30" s="36"/>
-      <c r="O30" s="36"/>
-      <c r="X30" s="43"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="35"/>
+      <c r="O30" s="35"/>
+      <c r="X30" s="42"/>
       <c r="Z30" s="17"/>
     </row>
     <row r="31" spans="1:26" ht="13.2" x14ac:dyDescent="0.3">
@@ -4469,7 +4722,7 @@
         <f>E31/34*35</f>
         <v>1965.1470588235295</v>
       </c>
-      <c r="G31" s="34" t="s">
+      <c r="G31" s="33" t="s">
         <v>110</v>
       </c>
       <c r="H31" s="16" t="s">
@@ -4490,14 +4743,14 @@
         <f t="shared" si="12"/>
         <v>5921.7470588235301</v>
       </c>
-      <c r="M31" s="37">
+      <c r="M31" s="36">
         <f>J33</f>
         <v>4519.7</v>
       </c>
-      <c r="N31" s="37" t="s">
+      <c r="N31" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="O31" s="36" t="str">
+      <c r="O31" s="35" t="str">
         <f>R31</f>
         <v>L4</v>
       </c>
@@ -4522,13 +4775,13 @@
         <f>R31</f>
         <v>L4</v>
       </c>
-      <c r="X31" s="43">
+      <c r="X31" s="42">
         <v>8.4</v>
       </c>
       <c r="Y31" s="16">
         <v>6</v>
       </c>
-      <c r="Z31" s="43">
+      <c r="Z31" s="42">
         <f t="shared" si="9"/>
         <v>8.3499005964214721</v>
       </c>
@@ -4554,7 +4807,7 @@
         <f>E32/34*35</f>
         <v>2724.8529411764707</v>
       </c>
-      <c r="G32" s="35" t="s">
+      <c r="G32" s="34" t="s">
         <v>111</v>
       </c>
       <c r="H32" s="16" t="s">
@@ -4575,14 +4828,14 @@
         <f t="shared" si="12"/>
         <v>6681.4529411764706</v>
       </c>
-      <c r="M32" s="40">
+      <c r="M32" s="39">
         <f>K33</f>
         <v>5716.2999999999993</v>
       </c>
-      <c r="N32" s="40" t="s">
+      <c r="N32" s="39" t="s">
         <v>84</v>
       </c>
-      <c r="O32" s="36" t="str">
+      <c r="O32" s="35" t="str">
         <f>R32</f>
         <v>L11</v>
       </c>
@@ -4607,13 +4860,13 @@
         <f>R32</f>
         <v>L11</v>
       </c>
-      <c r="X32" s="43">
+      <c r="X32" s="42">
         <v>8.4</v>
       </c>
       <c r="Y32" s="16">
         <v>6</v>
       </c>
-      <c r="Z32" s="43">
+      <c r="Z32" s="42">
         <f t="shared" si="9"/>
         <v>8.3499005964214721</v>
       </c>
@@ -4631,7 +4884,7 @@
       <c r="D33" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="E33" s="36">
+      <c r="E33" s="35">
         <f>(LEFT(B33,4)+RIGHT(B33,4))/2</f>
         <v>2278</v>
       </c>
@@ -4639,7 +4892,7 @@
         <f>E33/34*35</f>
         <v>2345</v>
       </c>
-      <c r="G33" s="35" t="s">
+      <c r="G33" s="34" t="s">
         <v>112</v>
       </c>
       <c r="H33" s="16" t="s">
@@ -4660,55 +4913,55 @@
         <f t="shared" si="12"/>
         <v>6301.6</v>
       </c>
-      <c r="M33" s="41">
+      <c r="M33" s="40">
         <f>L33</f>
         <v>6301.6</v>
       </c>
-      <c r="N33" s="41" t="s">
+      <c r="N33" s="40" t="s">
         <v>84</v>
       </c>
-      <c r="O33" s="36" t="str">
+      <c r="O33" s="35" t="str">
         <f>R33</f>
         <v>L14</v>
       </c>
-      <c r="P33" s="28">
+      <c r="P33" s="27">
         <f>L31</f>
         <v>5921.7470588235301</v>
       </c>
-      <c r="Q33" s="29" t="s">
+      <c r="Q33" s="28" t="s">
         <v>82</v>
       </c>
       <c r="R33" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="S33" s="28">
+      <c r="S33" s="27">
         <f>L32</f>
         <v>6681.4529411764706</v>
       </c>
-      <c r="T33" s="28" t="s">
+      <c r="T33" s="27" t="s">
         <v>83</v>
       </c>
       <c r="U33" s="16" t="str">
         <f>R33</f>
         <v>L14</v>
       </c>
-      <c r="X33" s="43">
+      <c r="X33" s="42">
         <v>8.4</v>
       </c>
       <c r="Y33" s="16">
         <v>6</v>
       </c>
-      <c r="Z33" s="43">
+      <c r="Z33" s="42">
         <f t="shared" si="9"/>
         <v>8.3499005964214721</v>
       </c>
     </row>
     <row r="34" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="X34" s="43"/>
+      <c r="X34" s="42"/>
       <c r="Z34" s="17"/>
     </row>
     <row r="35" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="X35" s="43"/>
+      <c r="X35" s="42"/>
       <c r="Z35" s="17"/>
     </row>
     <row r="36" spans="1:26" ht="12" x14ac:dyDescent="0.3">
@@ -4718,47 +4971,47 @@
       <c r="E36" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="F36" s="36">
+      <c r="F36" s="35">
         <f>F37</f>
         <v>4747.5</v>
       </c>
-      <c r="G36" s="36">
+      <c r="G36" s="35">
         <f>G37</f>
         <v>0.6</v>
       </c>
-      <c r="X36" s="43"/>
+      <c r="X36" s="42"/>
       <c r="Z36" s="17"/>
     </row>
     <row r="37" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="D37" s="32" t="s">
+      <c r="D37" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="E37" s="32" t="s">
+      <c r="E37" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="F37" s="32">
+      <c r="F37" s="31">
         <v>4747.5</v>
       </c>
-      <c r="G37" s="32">
+      <c r="G37" s="31">
         <v>0.6</v>
       </c>
-      <c r="X37" s="43"/>
+      <c r="X37" s="42"/>
       <c r="Z37" s="17"/>
     </row>
     <row r="38" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="D38" s="32" t="s">
+      <c r="D38" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="E38" s="32" t="s">
+      <c r="E38" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="F38" s="32">
+      <c r="F38" s="31">
         <v>4742</v>
       </c>
-      <c r="G38" s="32">
+      <c r="G38" s="31">
         <v>20</v>
       </c>
-      <c r="X38" s="43"/>
+      <c r="X38" s="42"/>
       <c r="Z38" s="17"/>
     </row>
     <row r="39" spans="1:26" ht="13.2" x14ac:dyDescent="0.3">
@@ -4794,21 +5047,21 @@
         <f>$F39+$F$36+7</f>
         <v>9186.1176470588234</v>
       </c>
-      <c r="M39" s="38">
+      <c r="M39" s="37">
         <f>MAX(I39:L39)</f>
         <v>9186.1176470588234</v>
       </c>
-      <c r="N39" s="38">
+      <c r="N39" s="37">
         <f>SQRT($H39^2+G$36^2)</f>
         <v>26.771430312347114</v>
       </c>
-      <c r="O39" s="39" t="s">
+      <c r="O39" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="P39" s="39" t="s">
+      <c r="P39" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="X39" s="43">
+      <c r="X39" s="42">
         <v>4.2</v>
       </c>
       <c r="Y39" s="16">

</xml_diff>